<commit_message>
Add AI Agent Report Excel report
</commit_message>
<xml_diff>
--- a/reports/agent-report.xlsx
+++ b/reports/agent-report.xlsx
@@ -447,7 +447,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>64143</t>
+          <t>64147</t>
         </is>
       </c>
     </row>
@@ -459,7 +459,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>11f53f99-df03-4073-8c00-d72e6554ece1</t>
+          <t>8cb0291a-8746-443e-a911-02123d8d69f7</t>
         </is>
       </c>
     </row>

</xml_diff>